<commit_message>
Chuẩn hoá đọc file word, PDF ==> Đang dự kiến sứa các loại file này thêo kiến trúc Gộp cả Excel thành 1 thể thống nhất
</commit_message>
<xml_diff>
--- a/hop/CongThuc_GiaVon.xlsx
+++ b/hop/CongThuc_GiaVon.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ThanhVu\kpht\KPHT_PMM\hop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38AA6222-E1C8-40FC-BC3F-2D2761FB9B59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{842429B4-C352-4412-BAAE-08D023A9C061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2160" yWindow="1485" windowWidth="17580" windowHeight="13995" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="44">
   <si>
     <r>
       <t>Nhập hàng và tính giá vốn</t>
@@ -270,6 +270,12 @@
   <si>
     <t>Ví đụ tuổi thu 61 tuổi bán 63 =&gt; {1-(61/63)}*100%= 3.175%</t>
   </si>
+  <si>
+    <t xml:space="preserve">OriginLabor +( GoldWeight * LossRate * GoldRate )+ TaxAmount + OtherCosts </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nhập trên phần </t>
+  </si>
 </sst>
 </file>
 
@@ -277,9 +283,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="169" formatCode="#,##0.000"/>
-    <numFmt numFmtId="171" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="172" formatCode="_(* #,##0.000_);_(* \(#,##0.000\);_(* &quot;-&quot;???_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="#,##0.000"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0.000_);_(* \(#,##0.000\);_(* &quot;-&quot;???_);_(@_)"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -416,9 +422,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="171" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -443,13 +449,13 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
+      <xdr:row>18</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
       <xdr:colOff>220165</xdr:colOff>
-      <xdr:row>49</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>162830</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -749,7 +755,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.28515625" customWidth="1"/>
@@ -900,68 +906,71 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
-        <v>36</v>
-      </c>
+      <c r="A16" s="6"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C18" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D21" s="9">
         <f>1-(61/63)</f>
         <v>3.1746031746031744E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="18" x14ac:dyDescent="0.25">
-      <c r="A21" s="8" t="s">
+    <row r="23" spans="1:9" ht="18" x14ac:dyDescent="0.25">
+      <c r="A23" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="G21">
+      <c r="G23">
         <f>1-(75/75.3)</f>
         <v>3.9840637450199168E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="6"/>
-      <c r="G22">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="6"/>
+      <c r="D24" t="s">
+        <v>42</v>
+      </c>
+      <c r="G24">
         <f>1-(61/63)</f>
         <v>3.1746031746031744E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="6"/>
-    </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -969,58 +978,70 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F27" s="10">
-        <v>33.746000000000002</v>
-      </c>
-      <c r="G27" s="11">
-        <v>16423000</v>
-      </c>
-      <c r="H27" s="12">
-        <f>F27*G27</f>
-        <v>554210558</v>
-      </c>
-      <c r="I27" s="12">
-        <f>H27*75/100</f>
-        <v>415657918.5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="6"/>
-      <c r="F28">
-        <v>25.3095</v>
-      </c>
-      <c r="G28" s="11">
-        <v>16423000</v>
-      </c>
-      <c r="H28" s="12">
-        <f>F28*G28</f>
-        <v>415657918.5</v>
-      </c>
-      <c r="I28" s="12">
-        <f>H28*75/100</f>
-        <v>311743438.875</v>
-      </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
+      </c>
+      <c r="F29" s="10">
+        <v>33.746000000000002</v>
+      </c>
+      <c r="G29" s="11">
+        <v>16423000</v>
+      </c>
+      <c r="H29" s="12">
+        <f>F29*G29</f>
+        <v>554210558</v>
+      </c>
+      <c r="I29" s="12">
+        <f>H29*75/100</f>
+        <v>415657918.5</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="6"/>
+      <c r="F30">
+        <v>25.3095</v>
+      </c>
+      <c r="G30" s="11">
+        <v>16423000</v>
+      </c>
+      <c r="H30" s="12">
+        <f>F30*G30</f>
+        <v>415657918.5</v>
+      </c>
+      <c r="I30" s="12">
+        <f>H30*75/100</f>
+        <v>311743438.875</v>
+      </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="6"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="6"/>
+      <c r="E34">
+        <f>1-(6)</f>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="7" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>